<commit_message>
fixed excel path for jenkins compatibility
</commit_message>
<xml_diff>
--- a/testdata/datafortesting.xlsx
+++ b/testdata/datafortesting.xlsx
@@ -467,11 +467,11 @@
         <v>180</v>
       </c>
       <c r="C2" t="n">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>failed</t>
         </is>
       </c>
     </row>
@@ -485,11 +485,11 @@
         <v>82</v>
       </c>
       <c r="C3" t="n">
-        <v>82</v>
+        <v>314</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>failed</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
         <v>349</v>
       </c>
       <c r="C6" t="n">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
         <v>128</v>
       </c>
       <c r="C8" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>

</xml_diff>